<commit_message>
Recompute expert agreement with correct reviewer files
Updated results:
- Cohen's kappa: 0.7618 (was 0.6231 with wrong files)
- Primary agreement: 294/380 (77.4%, was 64.1%)
- Exact match: 205/380 (53.9%, was 33.5%)
- Remaining discordances: 86 (was 136)
- All 380 questions now included (was 379)

Updated README and all output files.
</commit_message>
<xml_diff>
--- a/Question_Classification/results/expert_review/reviewer_confusion_matrix.xlsx
+++ b/Question_Classification/results/expert_review/reviewer_confusion_matrix.xlsx
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -564,7 +564,7 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="T2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2">
         <v>0</v>
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -650,7 +650,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -718,10 +718,10 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="X4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y4">
         <v>2</v>
@@ -956,7 +956,7 @@
         <v>0</v>
       </c>
       <c r="Y6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z6">
         <v>0</v>
@@ -965,7 +965,7 @@
         <v>0</v>
       </c>
       <c r="AB6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:28">
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1033,7 +1033,7 @@
         <v>0</v>
       </c>
       <c r="V7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7">
         <v>0</v>
@@ -1042,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="Y7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z7">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1086,7 +1086,7 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="Y8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z8">
         <v>0</v>
@@ -1145,7 +1145,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1214,13 +1214,13 @@
         <v>0</v>
       </c>
       <c r="Y9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z9">
         <v>0</v>
       </c>
       <c r="AA9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB9">
         <v>1</v>
@@ -1237,62 +1237,62 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>15</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
         <v>3</v>
       </c>
-      <c r="G10">
-        <v>2</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>11</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>1</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>6</v>
-      </c>
       <c r="W10">
         <v>0</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="Y10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z10">
         <v>0</v>
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1694,13 +1694,13 @@
         <v>1</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15">
         <v>0</v>
       </c>
       <c r="O15">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -1709,13 +1709,13 @@
         <v>0</v>
       </c>
       <c r="R15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15">
         <v>1</v>
       </c>
       <c r="T15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U15">
         <v>0</v>
@@ -1730,10 +1730,10 @@
         <v>1</v>
       </c>
       <c r="Y15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA15">
         <v>0</v>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="P16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q16">
         <v>0</v>
@@ -1967,7 +1967,7 @@
         <v>0</v>
       </c>
       <c r="R18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S18">
         <v>0</v>
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -2091,7 +2091,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -2130,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20">
         <v>0</v>
@@ -2145,13 +2145,13 @@
         <v>0</v>
       </c>
       <c r="T20">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="U20">
         <v>0</v>
       </c>
       <c r="V20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -2160,7 +2160,7 @@
         <v>1</v>
       </c>
       <c r="Y20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z20">
         <v>0</v>
@@ -2234,7 +2234,7 @@
         <v>0</v>
       </c>
       <c r="U21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V21">
         <v>0</v>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y21">
         <v>0</v>
@@ -2317,13 +2317,13 @@
         <v>0</v>
       </c>
       <c r="T22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U22">
         <v>0</v>
       </c>
       <c r="V22">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>1</v>
       </c>
       <c r="Z22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA22">
         <v>0</v>
@@ -2471,20 +2471,20 @@
         <v>0</v>
       </c>
       <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
         <v>2</v>
       </c>
-      <c r="O24">
-        <v>0</v>
-      </c>
-      <c r="P24">
-        <v>0</v>
-      </c>
-      <c r="Q24">
-        <v>0</v>
-      </c>
-      <c r="R24">
-        <v>3</v>
-      </c>
       <c r="S24">
         <v>0</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y24">
         <v>1</v>
@@ -2521,7 +2521,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -2590,7 +2590,7 @@
         <v>1</v>
       </c>
       <c r="Y25">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="Z25">
         <v>0</v>
@@ -2628,7 +2628,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -2667,7 +2667,7 @@
         <v>0</v>
       </c>
       <c r="V26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W26">
         <v>0</v>
@@ -2679,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="Z26">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="AA26">
         <v>0</v>
@@ -2747,7 +2747,7 @@
         <v>0</v>
       </c>
       <c r="T27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27">
         <v>0</v>
@@ -2768,7 +2768,7 @@
         <v>0</v>
       </c>
       <c r="AA27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB27">
         <v>0</v>
@@ -2857,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="AB28">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recompute expert agreement with correct (definitive) reviewer files
Final results:
- Cohen's kappa: 0.8557 (almost perfect agreement)
- Primary agreement: 328/380 (86.3%)
- Exact match: 254/380 (66.8%)
- Remaining discordances: 52
- Pipeline resolved: 95.9% (1208/1260)
</commit_message>
<xml_diff>
--- a/Question_Classification/results/expert_review/reviewer_confusion_matrix.xlsx
+++ b/Question_Classification/results/expert_review/reviewer_confusion_matrix.xlsx
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -668,7 +668,7 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -721,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>2</v>
       </c>
       <c r="Z4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA4">
         <v>0</v>
@@ -807,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>9</v>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6">
         <v>0</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1145,7 +1145,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1166,7 +1166,7 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -1199,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="T9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U9">
         <v>0</v>
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="AB9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:28">
@@ -1243,55 +1243,55 @@
         <v>0</v>
       </c>
       <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>16</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
         <v>2</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>15</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>1</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>3</v>
       </c>
       <c r="W10">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1383,7 +1383,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y11">
         <v>0</v>
@@ -1418,10 +1418,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -1442,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1510,7 +1510,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1611,7 +1611,7 @@
         <v>0</v>
       </c>
       <c r="N14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O14">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>0</v>
@@ -1700,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -1715,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15">
         <v>0</v>
@@ -1783,7 +1783,7 @@
         <v>0</v>
       </c>
       <c r="N16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16">
         <v>0</v>
@@ -1798,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="S16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T16">
         <v>0</v>
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="Z16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA16">
         <v>0</v>
@@ -2056,7 +2056,7 @@
         <v>0</v>
       </c>
       <c r="S19">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T19">
         <v>0</v>
@@ -2145,7 +2145,7 @@
         <v>0</v>
       </c>
       <c r="T20">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="U20">
         <v>0</v>
@@ -2157,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y20">
         <v>0</v>
@@ -2293,7 +2293,7 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22">
         <v>0</v>
@@ -2323,7 +2323,7 @@
         <v>0</v>
       </c>
       <c r="V22">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="Y22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z22">
         <v>0</v>
@@ -2341,7 +2341,7 @@
         <v>0</v>
       </c>
       <c r="AB22">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:28">
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y24">
         <v>1</v>
@@ -2524,7 +2524,7 @@
         <v>0</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -2536,10 +2536,10 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="S25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T25">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="X25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y25">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="Z25">
         <v>0</v>
@@ -2637,7 +2637,7 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26">
         <v>0</v>
@@ -2679,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="Z26">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AA26">
         <v>0</v>
@@ -2857,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="AB28">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>